<commit_message>
Ajustes de código y desarrollo del test 'LOGIN'.
</commit_message>
<xml_diff>
--- a/src/test/resources/data/registerData/registerData.xlsx
+++ b/src/test/resources/data/registerData/registerData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tomas\Desktop\Documents\Automation\ParaBank\src\test\resources\data\registerData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFB7C310-2A7B-43AE-A822-BC3713AE55FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C008CD99-B117-4F9B-A376-9B20E5AD4C09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1455" yWindow="2730" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3570" yWindow="4185" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="103">
   <si>
     <t>ID</t>
   </si>
@@ -331,6 +331,9 @@
   </si>
   <si>
     <t>FIRST_NAME_REQUIRED_ERROR;LAST_NAME_REQUIRED_ERROR;ADDRESS_REQUIRED_ERROR;CITY_REQUIRED_ERROR;STATE_REQUIRED_ERROR;ZIP_CODE_REQUIRED_ERROR;SSN_REQUIRED_ERROR;USERNAME_REQUIRED_ERROR;PASSWORD_REQUIRED_ERROR;PASSWORD_CONFIRM_REQUIRED_ERROR</t>
+  </si>
+  <si>
+    <t>PASSWORDS_MISMATCH_ERROR</t>
   </si>
 </sst>
 </file>
@@ -1271,6 +1274,9 @@
       <c r="L16">
         <v>12346</v>
       </c>
+      <c r="M16" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="20" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F20" s="2"/>

</xml_diff>